<commit_message>
docs: MVP completion plan sheet, corrections after the owner's answers
</commit_message>
<xml_diff>
--- a/Reports/MVP Completion Tasks.xlsx
+++ b/Reports/MVP Completion Tasks.xlsx
@@ -8,17 +8,19 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capstone scorecard" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner decisions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner actions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tasks" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capstone scorecard" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner decisions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner actions" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tasks'!$A$1:$H$42</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Capstone scorecard'!$A$1:$E$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Owner decisions'!$A$1:$D$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Owner actions'!$A$1:$B$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan'!$A$1:$I$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$H$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Capstone scorecard'!$A$1:$E$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Owner decisions'!$A$1:$D$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Owner actions'!$A$1:$B$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -40,7 +42,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -77,6 +79,31 @@
         <fgColor rgb="00C6E0B4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -90,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -98,16 +125,31 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -529,7 +571,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>1. AI feature: the capstone cases are AI cases. The app has one small AI feature (the Translate button via OpenRouter). The planned AI document check is not built. 2. Agentic-engineering evidence: there is no CLAUDE.md, and the .claude folder in the project is empty (no saved skill, slash command or subagent); GitHub shows no reviewed pull request. 3. Stack match: the criteria name Supabase; the project uses Neon (Postgres, row-level security, Neon Auth). This needs a one-line confirmation from the course lead. 4. A working live URL with the finished flow: the live site is behind the code (production runs the 31 October release), PR #47 must not go live before the app screens exist (see the release warning below), and the phone walk-through and a Stripe test payment have not been done by a person.</t>
+          <t>1. AI feature: the capstone cases are AI cases. The app has one small AI feature (the Translate button via OpenRouter). The planned AI document check is not built. 2. Agentic-engineering evidence: there is no CLAUDE.md, and the .claude folder in the project is empty (no saved skill, slash command or subagent); GitHub shows no reviewed pull request. 3. Stack match: the criteria name Supabase; the project uses Neon (Postgres, row-level security, Neon Auth). APPROVED by the owner on 1 November 2026; only the short evidence note remains. 4. A working live URL with the finished flow: the live site is behind the code (production runs the 31 October release), PR #47 must not go live before the app screens exist (see the release warning below), and the phone walk-through and a Stripe test payment have not been done by a person.</t>
         </is>
       </c>
     </row>
@@ -589,7 +631,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Tasks (sorted by importance) | Capstone scorecard (each criterion: met, partly, not met) | Owner decisions | Owner actions (dashboards and real-world steps).</t>
+          <t>Plan (the order to get everything done, phase by phase) | Tasks (sorted by importance) | Capstone scorecard | Owner decisions | Owner actions.</t>
         </is>
       </c>
     </row>
@@ -600,6 +642,1468 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>What happens</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Done when</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Needs first</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Who</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Effort</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Tasks sheet No</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Can run alongside</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>0.1</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>0 Decide and set up</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Hold PR #47 (do not merge): the server now requires a date and time on requests and the current app cannot send one.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>PR #47 stays open until step 1.9.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>everything</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>0 Decide and set up</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>AI feature planning session: choose the feature and the AI provider, write the design (questions in the chat reply of 1 Nov). Result: a written plan in docs/superpowers/plans/.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>AI plan approved by the owner.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>0.3, 1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>0.3</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>0 Decide and set up</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Add CLAUDE.md and the project .claude folder (project copies of the agents, commands and skills actually used, plus two new ones: /test-report and an RLS-check agent). Describe them in the README.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>CLAUDE.md in the root; .claude/ has at least 3 files; README section "How this project is built with Claude Code".</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>5, 6</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>0.2, 1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>0.4</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>0 Decide and set up</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Write the one-page RLS and auth evidence note (Neon approved by the owner).</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>docs/rls-and-auth-evidence.md.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>0.2, 1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>1 Finish Flow 1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Task 9: finish the notice wording (in-app, push, email, German and English) and correct the plan text.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Notice texts complete; i18n parity and notification specs pass.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>0.x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>1 Finish Flow 1</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Task 10a (app): ONE request form (what, where, date and time) with native date and time pickers (Finding 2). Remove the separate propose step for requests.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>A customer can send a request with a time on a phone build; jest tests for the form.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>3, 20</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>1 Finish Flow 1</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Task 10b (app): provider answer panel: quote with or without a date and time, switch "date and time confirmed", propose another time, reject.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Provider can answer every request type; jest tests.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>1 Finish Flow 1</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Task 10c (app): customer quote screen: Confirm; Decline with the offer to chat first; find another provider; pending-time confirm button; awaiting-time status text; no stand-in time shown; "discuss changes in the chat" instead of an edit button once a quote exists.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>The whole flow can be walked in the app; jest tests.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>1 Finish Flow 1</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Task 11 (app): "Quotes sent" and "My received quotes" on the account page, PDF open / download / print.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Both lists and the PDF open on a phone build.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>1 Finish Flow 1</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Task 12: retire the old proposed-booking path, make the time required in the contract, keep accept only for additional tasks.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>No second booking path; specs updated.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>1 Finish Flow 1</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Task 13: full suites once, test report in Reports/, README update, phone test script with a tap count before and after.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Reports/Flow-1-Test-Report.xlsx; all suites green.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>1.5, 1.6</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>1 Finish Flow 1</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Decide the open Flow 1 points (street privacy, second PDF, PDF language) and apply the answers.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Decisions recorded in the plan.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>1.2-1.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>1 Finish Flow 1</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Release: apply migrations 0024 to 0026 to kando-main, merge #47 and the app PR, check production, make a new Android build.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Production runs Flow 1; new APK installed on the test phone.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>1.7, 1.8, owner actions O.1</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>4, 34</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>1 Finish Flow 1</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Phone walk-through on Android with the test accounts, including a full Stripe TEST payment; fix what it finds; retest findings 4 and 6.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Walk-through list signed off by the owner; fixes merged.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>12, 20</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>2 AI feature</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Provider and data protection: choose the provider, sign the processing agreement, sign off the DPIA, add the key to Vercel (server side only).</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Provider contract and DPIA sign-off recorded in docs/legal-drafts.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>0.2</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>2, 25</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>2 AI feature</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Build the backend: table with row-level security for AI results, server job after upload, model call through the provider, result stored as a suggestion, rate limits and cost cap, tests (incl. a failing provider).</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Upload creates a suggestion; failures never block an upload; specs pass.</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>2.1, 0.2</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>2 AI feature</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Back office: a suggestion panel next to each document (type, name match, expiry, flags), staff decide as before; the decision is logged.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Reviewer sees suggestion and decides; admin specs pass.</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>2 AI feature</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Disclosure and privacy: label in German and English where the person uploads and where staff see the suggestion; privacy text names the provider; the Article 50 note.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Labels visible; docs/article-50-note.md.</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>2 AI feature</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Delete my data covers the AI result; export contains it.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Deletion spec proves removal.</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>2 AI feature</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Evaluation: run the feature on about 20 sample documents (made-up documents, never real ones), compare with the staff decision, record the result.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>A measured result (for example 18 of 20 correct) in Reports/.</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>3 Security and compliance</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Run the security scan on the final code (/security-scan and the three scanners); fix every critical and high finding and the open items (anonymous inserts into translations, owner_id readable, whole-row admin detail, server-only, CSP script-src).</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>docs/security-scan-&lt;date&gt;.md: no critical or high open.</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>1.7, 2.3</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>3.2</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>3 Security and compliance</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Secrets: scan working tree and history again; clean up Vercel Preview variables; mark secrets Sensitive; WAF rate-limit rules.</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Clean scan output; checklist ticked by the owner.</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>owner actions</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>3 Security and compliance</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Legal pages published (Impressum, Datenschutz, AGB, Ranking) in German and English; age and terms tick at sign-up; report this profile or photo; public web page to request deletion.</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Pages live; tick enforced; spec covers it.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>owner supplies company details</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>24, 11</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>2.x</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>3 Security and compliance</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Real deletion on the live Neon Auth with a throw-away account; confirm everything is gone.</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Written result in the evidence folder.</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>3 Security and compliance</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Run /code-review --comment on the release PR so the review is visible on GitHub; fix; the owner submits a GitHub review (Approve) and merges.</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>At least one PR shows a recorded review on GitHub.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>4 Quality and evidence</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Green repository: lint errors (38) and mobile type errors (4) fixed or excluded; CI green; update README "Where we are", Known gaps and test numbers.</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>pnpm lint, pnpm typecheck and CI all green on main.</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>23, 35</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>4 Quality and evidence</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Demo data on production: delete the old test accounts; create one demo customer and two published demo providers with approved documents, finished jobs and reviews.</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Demo walk-through works end to end on the live site.</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>1.9, 2.3</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>4 Quality and evidence</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>README top section: goal / problem / how it works paragraph, Situation-Complication-Resolution, stack, AI disclosure; re-check the scorecard sheet.</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Every row of the scorecard is Met.</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>all above</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>5 Presentation</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Deck in the SCR frame with the six points; screenshots and a recorded demo as fallback; evaluation numbers from the reports.</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Deck and demo script ready.</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>14, 26</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>5 Presentation</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Upload the project to showcase.turingcollege.com; rehearse the 10 minutes; prepare answers for the 5 minutes of questions (stack choice, RLS, AI risk, what is next).</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Showcase entry live; rehearsal done.</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>O.1</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Owner actions (run in parallel from day 1)</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Vercel Preview variables and plan, Stripe Preview webhooks, storage keys, Neon Auth settings, first administrator on production, Resend domain, FCM credentials (see the Owner actions sheet).</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Owner actions sheet ticked.</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>21, 33</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Phases 1 to 3</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I32"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -664,7 +2168,7 @@
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="10" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -686,7 +2190,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Not asked. Evidence exists in code and tests, not as a short note.</t>
+          <t>Neon APPROVED by the owner on 1 November 2026. Remaining: the one-page evidence note (RLS and auth) for the assessor.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -704,7 +2208,7 @@
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -736,7 +2240,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Both (owner decides provider and feature)</t>
+          <t>Both (owner decides provider and feature; planning started 1 Nov)</t>
         </is>
       </c>
     </row>
@@ -744,7 +2248,7 @@
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -784,7 +2288,7 @@
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -824,7 +2328,7 @@
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -864,7 +2368,7 @@
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -886,7 +2390,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Used in sessions only; nothing saved in the repo.</t>
+          <t>The agents, commands and plugin skills used live in the owner user folder (~/.claude) and in plugins, not in the project, so the repo shows none. Nothing saved in the project .claude folder.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -904,7 +2408,7 @@
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -926,7 +2430,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Review reports exist (PRs 14-16, 18-20, 46-47, assessment stages). No GitHub review recorded.</t>
+          <t>Reviews were done in Claude Code sessions and written up as Excel reports (PRs 14-16, 18-20, 46-47, assessment stages), but none is recorded ON GitHub (the API shows 0 reviews on 47 PRs; the 42 PRs with comments are mostly the Vercel bot). An assessor looking at GitHub sees no review.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -944,7 +2448,7 @@
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -984,7 +2488,7 @@
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1024,7 +2528,7 @@
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1064,7 +2568,7 @@
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1104,7 +2608,7 @@
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1144,7 +2648,7 @@
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1184,7 +2688,7 @@
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -1224,7 +2728,7 @@
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1264,7 +2768,7 @@
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1304,7 +2808,7 @@
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1344,7 +2848,7 @@
       <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1384,7 +2888,7 @@
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1424,7 +2928,7 @@
       <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1464,7 +2968,7 @@
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1504,7 +3008,7 @@
       <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1544,7 +3048,7 @@
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1584,7 +3088,7 @@
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1624,7 +3128,7 @@
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1664,7 +3168,7 @@
       <c r="A27" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -1704,7 +3208,7 @@
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1744,7 +3248,7 @@
       <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1784,7 +3288,7 @@
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1824,7 +3328,7 @@
       <c r="A31" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1864,7 +3368,7 @@
       <c r="A32" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1904,7 +3408,7 @@
       <c r="A33" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1944,7 +3448,7 @@
       <c r="A34" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -1984,7 +3488,7 @@
       <c r="A35" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2024,7 +3528,7 @@
       <c r="A36" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B36" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -2064,7 +3568,7 @@
       <c r="A37" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="6" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -2104,7 +3608,7 @@
       <c r="A38" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="6" t="inlineStr">
+      <c r="B38" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -2144,7 +3648,7 @@
       <c r="A39" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B39" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -2184,7 +3688,7 @@
       <c r="A40" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="6" t="inlineStr">
+      <c r="B40" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -2224,7 +3728,7 @@
       <c r="A41" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="6" t="inlineStr">
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -2264,7 +3768,7 @@
       <c r="A42" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="B42" s="7" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -2306,7 +3810,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2360,7 +3864,7 @@
           <t>Completeness and functionality; runs at a live Vercel URL or on a phone</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
@@ -2387,7 +3891,7 @@
           <t>User interface and interaction quality</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
@@ -2414,7 +3918,7 @@
           <t>Clear README.md with a goal / problem / how-it-works paragraph</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
@@ -2441,19 +3945,19 @@
           <t>Course stack: Next.js, Supabase Auth and RLS, Vercel</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Partly</t>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Met</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Next.js 16 and Vercel: yes. Supabase: no, Neon Postgres with row-level security and Neon Auth are used instead.</t>
+          <t>Next.js 16 and Vercel: yes. Neon Postgres with row-level security and Neon Auth instead of Supabase: approved by the owner (1 November 2026).</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Confirm with the course lead (task 1) and write the evidence note.</t>
+          <t>Write the evidence note (task 1).</t>
         </is>
       </c>
     </row>
@@ -2468,7 +3972,7 @@
           <t>CLAUDE.md</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>Not met</t>
         </is>
@@ -2495,7 +3999,7 @@
           <t>At least one skill, slash command or subagent used</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
@@ -2522,7 +4026,7 @@
           <t>At least one pull request reviewed before merging</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
@@ -2549,7 +4053,7 @@
           <t>Secrets out of the repo, server side only</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Met</t>
         </is>
@@ -2576,7 +4080,7 @@
           <t>Row-level security on every table holding user data</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr">
         <is>
           <t>Met</t>
         </is>
@@ -2603,7 +4107,7 @@
           <t>A /security-scan pass</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
@@ -2630,7 +4134,7 @@
           <t>AI-generated content disclosed (Article 50)</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
@@ -2657,7 +4161,7 @@
           <t>Working "delete my data" route (GDPR)</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
@@ -2684,7 +4188,7 @@
           <t>SCR or SMART framing, clear explanation</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>Not met</t>
         </is>
@@ -2711,7 +4215,7 @@
           <t>Showcase upload and 10 + 5 minute presentation</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>Not met</t>
         </is>
@@ -2733,7 +4237,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2974,7 +4478,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
docs: MVP completion tasks updated (AI decisions, .claude folder, review record plan, reuse map, reminders)
</commit_message>
<xml_diff>
--- a/Reports/MVP Completion Tasks.xlsx
+++ b/Reports/MVP Completion Tasks.xlsx
@@ -13,14 +13,18 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Capstone scorecard" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner decisions" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner actions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reminders" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reuse map" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan'!$A$1:$I$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan'!$A$1:$I$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$H$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Capstone scorecard'!$A$1:$E$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Owner decisions'!$A$1:$D$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Owner actions'!$A$1:$B$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Reminders'!$A$1:$D$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Reuse map'!$A$1:$D$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -520,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -554,89 +558,101 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Where the project stands</t>
+          <t>Latest update (1 November 2026, later)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>A large, working product: Expo phone app, Next.js website and back office on Vercel (https://skillweb.space), Neon Postgres with row-level security, Stripe Connect in TEST mode, invoices, chat, disputes, reviews, 4 cron jobs, German and English texts, 140+ commits, 47 pull requests, thousands of automated tests. Flow 1 (one request-to-booked flow with a quote document) is half built: the server side, the quote PDF, numbering and lists are done (PR #47, open, not merged); the app screens are not.</t>
+          <t>Owner decisions recorded: Neon approved; the AI feature uses an OpenRouter model, covers all documents including photo ID (sensitive data protected), automatic decisions are allowed with a human check in some cases, and the AI quote assistant is to be discussed when AI planning starts. The agents, commands and skills used in the project were added to the project .claude folder (branch chore/claude-folder, PR to be opened). The review finding was corrected: reviews were done and written up, but none is recorded on GitHub. A reuse map for the app screens was proposed (no new fields; the old preferredDate and accept screen fall away) and awaits the owner's confirmation. Reminders are saved (see the Reminders sheet).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>The four things that decide the assessment</t>
+          <t>Where the project stands</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>1. AI feature: the capstone cases are AI cases. The app has one small AI feature (the Translate button via OpenRouter). The planned AI document check is not built. 2. Agentic-engineering evidence: there is no CLAUDE.md, and the .claude folder in the project is empty (no saved skill, slash command or subagent); GitHub shows no reviewed pull request. 3. Stack match: the criteria name Supabase; the project uses Neon (Postgres, row-level security, Neon Auth). APPROVED by the owner on 1 November 2026; only the short evidence note remains. 4. A working live URL with the finished flow: the live site is behind the code (production runs the 31 October release), PR #47 must not go live before the app screens exist (see the release warning below), and the phone walk-through and a Stripe test payment have not been done by a person.</t>
+          <t>A large, working product: Expo phone app, Next.js website and back office on Vercel (https://skillweb.space), Neon Postgres with row-level security, Stripe Connect in TEST mode, invoices, chat, disputes, reviews, 4 cron jobs, German and English texts, 140+ commits, 47 pull requests, thousands of automated tests. Flow 1 (one request-to-booked flow with a quote document) is half built: the server side, the quote PDF, numbering and lists are done (PR #47, open, not merged); the app screens are not.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>RELEASE WARNING (act on this)</t>
+          <t>The four things that decide the assessment</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>PR #47 makes the server require a date and time on every new request (400 time-required without one). The current phone app and the production APK send requests without a time. If #47 is merged and deployed before Tasks 10 to 12 (the app screens), every new request from the existing app fails. Also: migrations 0024 to 0026 must be applied to the production database (kando-main) BEFORE the code that needs them is deployed (README rule). Recommended: keep #47 open until the app screens are ready, then merge and release together.</t>
+          <t>1. AI feature: the capstone cases are AI cases. The app has one small AI feature (the Translate button via OpenRouter). The planned AI document check is not built. 2. Agentic-engineering evidence: there is still no CLAUDE.md. The used agents, commands and skills are now in the project .claude folder (branch chore/claude-folder, not merged yet). Reviews were done in sessions and written up in Reports/, but GitHub records none: use /code-review --comment and a GitHub review before the next merge. 3. Stack match: the criteria name Supabase; the project uses Neon (Postgres, row-level security, Neon Auth). APPROVED by the owner on 1 November 2026; only the short evidence note remains. 4. A working live URL with the finished flow: the live site is behind the code (production runs the 31 October release), PR #47 must not go live before the app screens exist (see the release warning below), and the phone walk-through and a Stripe test payment have not been done by a person.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Recommended order of work</t>
+          <t>RELEASE WARNING (act on this)</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Phase 1 (finish the product): Flow 1 Tasks 9 to 13, owner decisions that block it, merge and release with migrations, phone walk-through. Phase 2 (the AI feature): decide the provider, build the AI document check with disclosure. Phase 3 (assessment evidence): CLAUDE.md, a project skill/command/subagent, a reviewed PR, security scan and fixes, README paragraph, GDPR and Article 50 checks. Phase 4 (presentation): demo accounts, deck in the SCR frame, showcase upload, rehearsal.</t>
+          <t>PR #47 makes the server require a date and time on every new request (400 time-required without one). The current phone app and the production APK send requests without a time. If #47 is merged and deployed before Tasks 10 to 12 (the app screens), every new request from the existing app fails. Also: migrations 0024 to 0026 must be applied to the production database (kando-main) BEFORE the code that needs them is deployed (README rule). Recommended: keep #47 open until the app screens are ready, then merge and release together.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Not needed for the capstone</t>
+          <t>Recommended order of work</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>App Store and Google Play submission, real payments (live Stripe keys), the lawyer and tax answers for real money, Flow 2 (availability and instant booking) and the post-launch feature list. They stay documented so nothing is lost, but they are marked Low or Medium on the Tasks sheet. The capstone accepts a phone or emulator build; Android works today (iPhone needs a paid Apple Developer account).</t>
+          <t>Phase 1 (finish the product): Flow 1 Tasks 9 to 13, owner decisions that block it, merge and release with migrations, phone walk-through. Phase 2 (the AI feature): decide the provider, build the AI document check with disclosure. Phase 3 (assessment evidence): CLAUDE.md, a project skill/command/subagent, a reviewed PR, security scan and fixes, README paragraph, GDPR and Article 50 checks. Phase 4 (presentation): demo accounts, deck in the SCR frame, showcase upload, rehearsal.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Effort scale</t>
+          <t>Not needed for the capstone</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>S = up to half a day, M = one to two days, L = three days or more (one working session of Claude Code plus owner input where stated). Who: Claude = can be built or written in a session; Owner = a decision, a dashboard action or a real-world step only the owner can do; Both = needs the owner's input first.</t>
+          <t>App Store and Google Play submission, real payments (live Stripe keys), the lawyer and tax answers for real money, Flow 2 (availability and instant booking) and the post-launch feature list. They stay documented so nothing is lost, but they are marked Low or Medium on the Tasks sheet. The capstone accepts a phone or emulator build; Android works today (iPhone needs a paid Apple Developer account).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>Effort scale</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>S = up to half a day, M = one to two days, L = three days or more (one working session of Claude Code plus owner input where stated). Who: Claude = can be built or written in a session; Owner = a decision, a dashboard action or a real-world step only the owner can do; Both = needs the owner's input first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>Sheets</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Plan (the order to get everything done, phase by phase) | Tasks (sorted by importance) | Capstone scorecard | Owner decisions | Owner actions.</t>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Plan (the order to get everything done, phase by phase) | Tasks (sorted by importance) | Capstone scorecard | Owner decisions | Owner actions | Reminders | Reuse map (app screens and fields).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B9"/>
+  <autoFilter ref="A1:B10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -647,7 +663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -768,7 +784,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>AI feature planning session: choose the feature and the AI provider, write the design (questions in the chat reply of 1 Nov). Result: a written plan in docs/superpowers/plans/.</t>
+          <t>AI feature planning: the owner decisions are in (OpenRouter model; all documents including photo ID, sensitive data protected; automatic decisions with a human check in some cases). Still to settle in the plan: the human-check rule, how ID data is protected, the model, cost cap, and the AI quote assistant (owner asked to be reminded). Result: a written plan in docs/superpowers/plans/.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -815,12 +831,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Add CLAUDE.md and the project .claude folder (project copies of the agents, commands and skills actually used, plus two new ones: /test-report and an RLS-check agent). Describe them in the README.</t>
+          <t>PARTLY DONE: the .claude folder with the used agents, commands and skills and its README is on branch chore/claude-folder (open the PR, review it with /code-review --comment, owner approves on GitHub, merge). Still to do: CLAUDE.md in the root, the /test-report command, the RLS-check agent, and a README section "How this project is built with Claude Code".</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>CLAUDE.md in the root; .claude/ has at least 3 files; README section "How this project is built with Claude Code".</t>
+          <t>CLAUDE.md in the root; .claude merged to main; README section added.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -830,7 +846,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Both</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -840,7 +856,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>5, 6</t>
+          <t>5, 6, 7</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -897,24 +913,24 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>1.1</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>1 Finish Flow 1</t>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>0 Decide and set up</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Task 9: finish the notice wording (in-app, push, email, German and English) and correct the plan text.</t>
+          <t>Confirm the reuse map for the app screens (Reuse map sheet) and the decision to keep direct booking until Flow 2; then update Tasks 10 to 12 of the Flow 1 plan as a reuse map (plan text only).</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Notice texts complete; i18n parity and notification specs pass.</t>
+          <t>Owner confirmation; plan updated.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -924,72 +940,76 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>3, 17, 28</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>0.2, 0.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>0 Decide and set up</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Post a Review record comment on each merged PR that has a written review (owner go-ahead pending).</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Comments visible on the merged PRs.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>owner go-ahead</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
           <t>Claude</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>0.x</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>1.2</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>1 Finish Flow 1</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Task 10a (app): ONE request form (what, where, date and time) with native date and time pickers (Finding 2). Remove the separate propose step for requests.</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>A customer can send a request with a time on a phone build; jest tests for the form.</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>1.1</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>3, 20</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr"/>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>everything</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -999,17 +1019,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Task 10b (app): provider answer panel: quote with or without a date and time, switch "date and time confirmed", propose another time, reject.</t>
+          <t>Task 9: finish the notice wording (in-app, push, email, German and English) and correct the plan text.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Provider can answer every request type; jest tests.</t>
+          <t>Notice texts complete; i18n parity and notification specs pass.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1019,20 +1039,24 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr"/>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>0.x</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1042,17 +1066,17 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Task 10c (app): customer quote screen: Confirm; Decline with the offer to chat first; find another provider; pending-time confirm button; awaiting-time status text; no stand-in time shown; "discuss changes in the chat" instead of an edit button once a quote exists.</t>
+          <t>Task 10a (app): ONE request form by extracting the shared "when and where" fields from TimeProposalForm (date, time, duration, on site, address prefilled from the saved account address, note) with native date and time pickers (Finding 2); remove the old preferredDate field from the form. The same shared fields serve the enter-a-time and counter screens.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>The whole flow can be walked in the app; jest tests.</t>
+          <t>A customer can send a request with a time on a phone build; jest tests for the form.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1067,7 +1091,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3, 20</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
@@ -1075,7 +1099,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>1.5</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -1085,17 +1109,17 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Task 11 (app): "Quotes sent" and "My received quotes" on the account page, PDF open / download / print.</t>
+          <t>Task 10b (app): provider answer panel by extending the existing SendQuoteForm (amount, scope, optional date, time, duration) with the switch "date and time confirmed", prefilled with the request's time; propose another time; reject (decline already exists).</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Both lists and the PDF open on a phone build.</t>
+          <t>Provider can answer every request type; jest tests.</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1110,19 +1134,15 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>16</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>1.6</t>
-        </is>
-      </c>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -1132,17 +1152,17 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Task 12: retire the old proposed-booking path, make the time required in the contract, keep accept only for additional tasks.</t>
+          <t>Task 10c (app): customer quote screen by extending the existing QuoteCard and request page: Confirm (replaces the accept screen, which falls away); Decline with the offer to chat first; find another provider; pending-time confirm button; awaiting-time status text; no stand-in time shown; "discuss changes in the chat" instead of an edit button once a quote exists.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>No second booking path; specs updated.</t>
+          <t>The whole flow can be walked in the app; jest tests.</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>1.4</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1157,19 +1177,15 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>1.5</t>
-        </is>
-      </c>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>1.7</t>
+          <t>1.5</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -1179,17 +1195,17 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Task 13: full suites once, test report in Reports/, README update, phone test script with a tap count before and after.</t>
+          <t>Task 11 (app): "Quotes sent" and "My received quotes" on the account page, PDF open / download / print.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Reports/Flow-1-Test-Report.xlsx; all suites green.</t>
+          <t>Both lists and the PDF open on a phone build.</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>1.5, 1.6</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1204,15 +1220,19 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1222,44 +1242,44 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Decide the open Flow 1 points (street privacy, second PDF, PDF language) and apply the answers.</t>
+          <t>Task 12: retire the old proposed-booking path for quotes, make the time required in the contract, delete preferredDate use and the AcceptQuoteScreen route, keep accept only for additional tasks; KEEP direct booking until Flow 2.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Decisions recorded in the plan.</t>
+          <t>No second booking path; specs updated.</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1.4</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>17</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>1.2-1.7</t>
+          <t>1.5</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>1.7</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1269,22 +1289,22 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Release: apply migrations 0024 to 0026 to kando-main, merge #47 and the app PR, check production, make a new Android build.</t>
+          <t>Task 13: full suites once, test report in Reports/, README update, phone test script with a tap count before and after.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Production runs Flow 1; new APK installed on the test phone.</t>
+          <t>Reports/Flow-1-Test-Report.xlsx; all suites green.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>1.7, 1.8, owner actions O.1</t>
+          <t>1.5, 1.6</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1294,7 +1314,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>4, 34</t>
+          <t>18</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
@@ -1302,132 +1322,132 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>1 Finish Flow 1</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Decide the open Flow 1 points (street privacy, second PDF, PDF language) and apply the answers.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Decisions recorded in the plan.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>1.2-1.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>1 Finish Flow 1</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Release: apply migrations 0024 to 0026 to kando-main, merge #47 and the app PR, check production, make a new Android build.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Production runs Flow 1; new APK installed on the test phone.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>1.7, 1.8, owner actions O.1</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>4, 34</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
           <t>1.10</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>1 Finish Flow 1</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Phone walk-through on Android with the test accounts, including a full Stripe TEST payment; fix what it finds; retest findings 4 and 6.</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Walk-through list signed off by the owner; fixes merged.</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>1.9</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>12, 20</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>2.1</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>2 AI feature</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Provider and data protection: choose the provider, sign the processing agreement, sign off the DPIA, add the key to Vercel (server side only).</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Provider contract and DPIA sign-off recorded in docs/legal-drafts.</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>0.2</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>2, 25</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Phase 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>2.2</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>2 AI feature</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Build the backend: table with row-level security for AI results, server job after upload, model call through the provider, result stored as a suggestion, rate limits and cost cap, tests (incl. a failing provider).</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Upload creates a suggestion; failures never block an upload; specs pass.</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>2.1, 0.2</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
@@ -1435,7 +1455,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -1445,40 +1465,44 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Back office: a suggestion panel next to each document (type, name match, expiry, flags), staff decide as before; the decision is logged.</t>
+          <t>Provider and data protection: choose the provider, sign the processing agreement, sign off the DPIA, add the key to Vercel (server side only).</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Reviewer sees suggestion and decides; admin specs pass.</t>
+          <t>Provider contract and DPIA sign-off recorded in docs/legal-drafts.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>0.2</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Claude</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>S</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr"/>
+          <t>2, 25</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>2.4</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1488,17 +1512,17 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Disclosure and privacy: label in German and English where the person uploads and where staff see the suggestion; privacy text names the provider; the Article 50 note.</t>
+          <t>Build the backend: table with row-level security for AI results, server job after upload, model call through the provider, result stored as a suggestion, rate limits and cost cap, tests (incl. a failing provider).</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Labels visible; docs/article-50-note.md.</t>
+          <t>Upload creates a suggestion; failures never block an upload; specs pass.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>2.3</t>
+          <t>2.1, 0.2</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1508,12 +1532,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>L</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
@@ -1521,7 +1545,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1531,12 +1555,12 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Delete my data covers the AI result; export contains it.</t>
+          <t>Back office: a suggestion panel next to each document (type, name match, expiry, flags), staff decide as before; the decision is logged.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Deletion spec proves removal.</t>
+          <t>Reviewer sees suggestion and decides; admin specs pass.</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1551,161 +1575,153 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>2.3</t>
-        </is>
-      </c>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>2 AI feature</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Disclosure and privacy: label in German and English where the person uploads and where staff see the suggestion; privacy text names the provider; the Article 50 note.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Labels visible; docs/article-50-note.md.</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>2 AI feature</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Delete my data covers the AI result; export contains it.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Deletion spec proves removal.</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>2 AI feature</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Evaluation: run the feature on about 20 sample documents (made-up documents, never real ones), compare with the staff decision, record the result.</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>A measured result (for example 18 of 20 correct) in Reports/.</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>3.1</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="inlineStr">
-        <is>
-          <t>3 Security and compliance</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Run the security scan on the final code (/security-scan and the three scanners); fix every critical and high finding and the open items (anonymous inserts into translations, owner_id readable, whole-row admin detail, server-only, CSP script-src).</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>docs/security-scan-&lt;date&gt;.md: no critical or high open.</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>1.7, 2.3</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>3.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>3.2</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>3 Security and compliance</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Secrets: scan working tree and history again; clean up Vercel Preview variables; mark secrets Sensitive; WAF rate-limit rules.</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Clean scan output; checklist ticked by the owner.</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>owner actions</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>3.1</t>
-        </is>
-      </c>
+      <c r="I23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1715,22 +1731,22 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Legal pages published (Impressum, Datenschutz, AGB, Ranking) in German and English; age and terms tick at sign-up; report this profile or photo; public web page to request deletion.</t>
+          <t>Run the security scan on the final code (/security-scan and the three scanners); fix every critical and high finding and the open items (anonymous inserts into translations, owner_id readable, whole-row admin detail, server-only, CSP script-src).</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Pages live; tick enforced; spec covers it.</t>
+          <t>docs/security-scan-&lt;date&gt;.md: no critical or high open.</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>owner supplies company details</t>
+          <t>1.7, 2.3</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Both</t>
+          <t>Claude</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1740,19 +1756,19 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>24, 11</t>
+          <t>8</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>2.x</t>
+          <t>3.2</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>3.2</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
@@ -1762,17 +1778,17 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Real deletion on the live Neon Auth with a throw-away account; confirm everything is gone.</t>
+          <t>Secrets: scan working tree and history again; clean up Vercel Preview variables; mark secrets Sensitive; WAF rate-limit rules.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Written result in the evidence folder.</t>
+          <t>Clean scan output; checklist ticked by the owner.</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>1.9</t>
+          <t>owner actions</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1787,136 +1803,144 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr"/>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
+          <t>3.3</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>3 Security and compliance</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Legal pages published (Impressum, Datenschutz, AGB, Ranking) in German and English; age and terms tick at sign-up; report this profile or photo; public web page to request deletion.</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Pages live; tick enforced; spec covers it.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>owner supplies company details</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>24, 11</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>2.x</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>3 Security and compliance</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Real deletion on the live Neon Auth with a throw-away account; confirm everything is gone.</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Written result in the evidence folder.</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>3 Security and compliance</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>Run /code-review --comment on the release PR so the review is visible on GitHub; fix; the owner submits a GitHub review (Approve) and merges.</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>At least one PR shows a recorded review on GitHub.</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>1.7</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>7</t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>4.1</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>4 Quality and evidence</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Green repository: lint errors (38) and mobile type errors (4) fixed or excluded; CI green; update README "Where we are", Known gaps and test numbers.</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>pnpm lint, pnpm typecheck and CI all green on main.</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>1.9</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Claude</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>23, 35</t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>4.2</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>4 Quality and evidence</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Demo data on production: delete the old test accounts; create one demo customer and two published demo providers with approved documents, finished jobs and reviews.</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Demo walk-through works end to end on the live site.</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>1.9, 2.3</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>22</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
@@ -1924,181 +1948,267 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>4 Quality and evidence</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Green repository: lint errors (38) and mobile type errors (4) fixed or excluded; CI green; update README "Where we are", Known gaps and test numbers.</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>pnpm lint, pnpm typecheck and CI all green on main.</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>23, 35</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>4 Quality and evidence</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Demo data on production: delete the old test accounts; create one demo customer and two published demo providers with approved documents, finished jobs and reviews.</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Demo walk-through works end to end on the live site.</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>1.9, 2.3</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
           <t>4.3</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>4 Quality and evidence</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>README top section: goal / problem / how it works paragraph, Situation-Complication-Resolution, stack, AI disclosure; re-check the scorecard sheet.</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Every row of the scorecard is Met.</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>all above</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>Claude</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>5 Presentation</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Deck in the SCR frame with the six points; screenshots and a recorded demo as fallback; evaluation numbers from the reports.</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Deck and demo script ready.</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Both</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>14, 26</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>5 Presentation</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>Upload the project to showcase.turingcollege.com; rehearse the 10 minutes; prepare answers for the 5 minutes of questions (stack choice, RLS, AI risk, what is next).</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Showcase entry live; rehearsal done.</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="9" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
         <is>
           <t>O.1</t>
         </is>
       </c>
-      <c r="B32" s="9" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>Owner actions (run in parallel from day 1)</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Vercel Preview variables and plan, Stripe Preview webhooks, storage keys, Neon Auth settings, first administrator on production, Resend domain, FCM credentials (see the Owner actions sheet).</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Owner actions sheet ticked.</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>21, 33</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>Phases 1 to 3</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I32"/>
+  <autoFilter ref="A1:I34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2180,7 +2290,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Confirm with the course lead (STL) that Neon (Postgres, row-level security, Neon Auth/Better Auth) is accepted in place of Supabase. Ask in writing and keep the answer. Prepare a one-page "RLS and auth evidence" note: every table holding user data is classified in packages/db/src/rls.ts and a check lists any table that is not; the policies, triggers and role split (app_user vs owner) are tested by the integration specs.</t>
+          <t>Confirm with the course lead (STL) that Neon [DONE: approved by the owner 1 Nov 2026; only the evidence note remains] (Postgres, row-level security, Neon Auth/Better Auth) is accepted in place of Supabase. Ask in writing and keep the answer. Prepare a one-page "RLS and auth evidence" note: every table holding user data is classified in packages/db/src/rls.ts and a check lists any table that is not; the policies, triggers and role split (app_user vs owner) are tested by the integration specs.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -2220,7 +2330,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Decide and build the capstone AI feature. Recommended: AI check of uploaded verification documents. A vision-capable model (via OpenRouter, server side only) reads the uploaded document, suggests its type, name match and expiry date, and flags problems; the result is stored per document (row-level security), shown to staff as a SUGGESTION in the back office; staff still decide. Fits the existing documents flow, the planned DPIA (docs/legal-drafts/dpia-ai-document-checks-draft.md) and the "multi-modal" case. Build: server job after upload, table with RLS, back-office panel, German and English disclosure text, tests, a "delete my data" path that removes the AI result. Alternatives if the owner prefers: AI help in the chat contact check, or an AI "quote assistant" that drafts the scope text of a quote from the request.</t>
+          <t>Decide and build the capstone AI feature. Agreed direction: AI check of uploaded verification documents, ALL document types including photo ID. A vision-capable OpenRouter model (server side only) reads the uploaded document, suggests its type, name match and expiry date, and flags problems; the result is stored per document (row-level security). Automatic decisions are allowed, but a human checks some cases (rule to design: for example low confidence, every ID photo, a name mismatch, a random sample). ID data is protected: visible only to the person and staff, never logged, sent to the model only for the check, deleted with the account. Fits the existing documents flow, the planned DPIA (docs/legal-drafts/dpia-ai-document-checks-draft.md) and the "multi-modal" case. Build: server job after upload, table with RLS, back-office panel, German and English disclosure text, tests, a "delete my data" path that removes the AI result. Alternatives if the owner prefers: AI help in the chat contact check, or an AI "quote assistant" that drafts the scope text of a quote from the request.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -2230,7 +2340,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Planned in the README ("AI document checks") but not built. DPIA is a draft. The AI provider is undecided (recommendation Mistral; needs EU data location, a processing agreement, no training on the data).</t>
+          <t>Owner decisions 1 Nov 2026: an OpenRouter model must be used; all documents including photo ID (the sensitive ID data must be protected); automatic decisions allowed, checked by a human in some cases; the AI quote assistant is to be discussed at AI planning (reminder saved). Not built. DPIA is a draft; EU data location, processing terms and no-training settings must still be checked for the chosen OpenRouter model.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -2260,7 +2370,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Finish Flow 1 in the app (Task 10): ONE request form (what, where, date and time); the provider answer panel (quote with or without a time, switch "date and time confirmed", reject); the customer quote screen (confirm, decline with the offer to chat first, find another provider); pending-time display and confirm button (pendingTime is in the contract); the awaiting-time status text and hiding the stand-in time; "discuss changes in the chat" instead of an edit button once a quote exists; date and time pickers (Finding 2).</t>
+          <t>Finish Flow 1 in the app (Task 10), by REUSING the existing screens and fields (see the Reuse map sheet; owner confirmation pending): ONE request form (what, where, date and time); the provider answer panel (quote with or without a time, switch "date and time confirmed", reject); the customer quote screen (confirm, decline with the offer to chat first, find another provider); pending-time display and confirm button (pendingTime is in the contract); the awaiting-time status text and hiding the stand-in time; "discuss changes in the chat" instead of an edit button once a quote exists; date and time pickers (Finding 2).</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -2390,7 +2500,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>The agents, commands and plugin skills used live in the owner user folder (~/.claude) and in plugins, not in the project, so the repo shows none. Nothing saved in the project .claude folder.</t>
+          <t>PARTLY DONE 1 Nov 2026: the verified agents (ai-architect, ai-researcher, ai-code-reviewer, nextjs- and vercel-security-scanner), the commands security-scan and security-scan-changed and the skills brainstorming, writing-plans, subagent-driven-development and neon-postgres are copied into the project .claude folder with a README (branch chore/claude-folder, commit ed55d72, PR to open). Still to add: a /test-report command and an RLS-check agent, and use each once.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -2420,7 +2530,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Have at least one pull request reviewed before it is merged, visibly on GitHub: run /code-review --comment on the next PR (inline comments), fix the findings, then the owner submits a GitHub review (Approve) and merges. Keep the review reports (Reports/PRs-46-47-Review-Report.xlsx is the model).</t>
+          <t>Have at least one pull request reviewed before it is merged, visibly on GitHub: run /code-review --comment on the next PR (inline comments), fix the findings, then the owner submits a GitHub review (Approve) and merges. Good first candidate: the .claude folder PR. In addition, post a "Review record" comment on each merged PR that has a written review (14 to 16, 18 to 20, 46, 47, the assessment-fix PRs) with the findings and fixes; owner go-ahead pending (comments post under the owner GitHub account; nothing is invented for PRs without a written review). Reminder saved for every merge.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -2820,7 +2930,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Task 12: retire the old proposed-booking path and make the time required in the contract (RequestInputSchema). Keep /quotes/[id]/accept for additional tasks only. Check that nothing else uses POST /bookings (direct booking, seed, mobile api).</t>
+          <t>Task 12: retire the old proposed-booking path FOR QUOTES and make the time required in the contract (RequestInputSchema); remove the old preferredDate field from the app form (the database column stays for old requests until now) and the AcceptQuoteScreen route. Keep /quotes/[id]/accept for additional tasks only. KEEP direct booking (POST /bookings, the Book button for fixed-price services) until Flow 2 replaces it: two ways to propose a time on a booking exist knowingly until then.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -3260,7 +3370,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Task 14 (optional): a "Needs your answer" list on Home for the pop-out item that was replaced; also reconsider the open items from the phone test (job disappears after notification).</t>
+          <t>Task 14 (optional) and the inbox (finding 5) are ONE list, not two: build "Needs your answer" on Home as the first version of the inbox, so the same information is not built twice.</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -4006,12 +4116,12 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Used in sessions (code-review, security scanners, research/review subagents, plan skills) but nothing saved in the repo (.claude is empty).</t>
+          <t>Used in sessions and now saved in the project .claude folder with a README (branch chore/claude-folder, not merged yet). CLAUDE.md still missing.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Task 6.</t>
+          <t>Tasks 5, 6.</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4143,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Owner merges every PR after CI and reports exist; GitHub shows no formal review.</t>
+          <t>Reviews were done in sessions and written up in Reports/; GitHub records none (0 reviews on 47 PRs). Review records on merged PRs and a GitHub review on the next PR are planned.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -4639,4 +4749,486 @@
   <autoFilter ref="A1:B12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>What</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Who reminds</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Before every merge</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Run /code-review --comment on the PR, fix the findings, and submit a GitHub review (Approve) in the PR page BEFORE merging. At least for the next release PR (the capstone needs a reviewed PR visible on GitHub).</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Claude reminds at each PR</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Saved (memory)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>AI planning</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Discuss the AI quote assistant (drafts the quote text from a request) when the AI feature planning starts.</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Claude reminds at AI planning</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Saved (memory)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Before the demo</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Street privacy question: the street is stored in the request and hidden only in the responses. Accept for the MVP or move it into a protected place?</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Claude raises it after Task 10</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Saved (memory)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Stand-in start time for awaiting-time bookings (nullable start_at, or filter on status). Documented in the README Known gaps.</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Claude raises it after the capstone</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>In README</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Plan</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>AI document check: define the human-check rule and the ID-data protection before building.</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>At AI planning</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Reply on the reuse map, direct booking kept until Flow 2, review records on merged PRs, and opening the PR for the .claude folder.</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Waiting for the owner</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Screen or field</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Exists today</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Reuse / change</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Falls away or stays as a known duplicate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Request form (customer)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>description, preferredDate (day only, typed), photos</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>KEEP description and photos; ADD the shared when-and-where fields (reuse TimeProposalForm: date, time, duration, on site, address, note) with native pickers; address prefilled from the saved account address</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>preferredDate (stop sending it now; the database column and its display stay for old requests until Task 12)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Shared "when and where" fields</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>TimeProposalForm: date, time, duration, on site, address, note (used by Book, Accept quote and Counter)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>ONE shared component, extracted and given native pickers; used by the request form, the enter-a-time screen and the counter</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Nothing duplicated: no second set of fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Provider answer (quote)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>SendQuoteForm: amount, scope, suggested date, time, duration</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>KEEP and extend: date, time, duration become optional with the switch "date and time confirmed", prefilled from the request; reject exists already (decline)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>The "suggestion" label and its text key</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Customer quote card</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>QuoteCard: amount, scope, suggested time, status, validity, Accept button</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>KEEP; button becomes Confirm (direct call, no time entry); add the quote number, revision, "date and time to be confirmed" and later the PDF link</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>The navigation to the accept screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Accept quote screen</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>AcceptQuoteScreen and /bookings/accept (customer proposes a time after a quote)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>FALLS AWAY (the customer confirms; the time is in the request and the quote). Server route /quotes/[id]/accept stays for additional tasks</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Request page</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>request-detail: description, preferredDate, quotes, withdraw/decline</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>KEEP; show time and place; "discuss changes in the chat" instead of editing once a quote exists; Decline offers the chat first; find another provider</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>preferredDate display (old requests only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Booking page</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>booking-detail with pay, cancel, finish, counter sheet (PR 45)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>KEEP; add the pending-time block with a confirm button and the awaiting-time text (stand-in time never shown); reuse the OpenChat + enter-time pattern from the counter sheet</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Nothing</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Counter screen</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>CounterScreen (counter a proposed booking time)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>KEEP for direct bookings; the enter-a-time screen for awaiting-time is the SAME screen with another submit call</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>No separate form</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Direct booking</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>BookScreen and POST /bookings for fixed-price services</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>KEEP until Flow 2 (instant booking) replaces it</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Two ways to propose a time on a booking coexist knowingly (proposed/counter vs awaiting-time/pending time); unify in Flow 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Quote lists (Task 11)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>New: Quotes sent / My received quotes on the account page</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>List rows open the EXISTING request page; PDF link on the row</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>No new detail screen</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Inbox / Needs your answer (Task 14, finding 5)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Notices on Home and My bookings</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>ONE list: build Needs your answer as the first version of the inbox</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>No separate pop-out or second list</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Server fields</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>requests.start_at, duration_min, on_site, address, note; quotes.start_at, duration_min; bookings.start_at and pending-time columns</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>All already built and shared through the TimeProposal shape; nothing new to add for the screens</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>preferredDate in the contract input after old app builds are gone (Task 12)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D13"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: remove the old preferredDate field everywhere (column dropped, contract, server, export, app, texts); report updated
</commit_message>
<xml_diff>
--- a/Reports/MVP Completion Tasks.xlsx
+++ b/Reports/MVP Completion Tasks.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Owner decisions recorded: Neon approved; the AI feature uses an OpenRouter model, covers all documents including photo ID (sensitive data protected), automatic decisions are allowed with a human check in some cases, and the AI quote assistant is to be discussed when AI planning starts. The agents, commands and skills used in the project were added to the project .claude folder (branch chore/claude-folder, PR to be opened). The review finding was corrected: reviews were done and written up, but none is recorded on GitHub. A reuse map for the app screens was proposed (no new fields; the old preferredDate and accept screen fall away) and awaits the owner's confirmation. Reminders are saved (see the Reminders sheet).</t>
+          <t>Owner decisions recorded: Neon approved; the AI feature uses an OpenRouter model, covers all documents including photo ID (sensitive data protected), automatic decisions are allowed with a human check in some cases, and the AI quote assistant is to be discussed when AI planning starts. The agents, commands and skills used in the project were added to the project .claude folder (branch chore/claude-folder, PR to be opened). The review finding was corrected: reviews were done and written up, but none is recorded on GitHub. preferredDate was removed completely (database column, contract, server, export, app form and display, texts; migration 0027) because nobody uses the app; a scan found no other unused table or column (currencies.minor_units is kept for other currencies). A reuse map for the app screens was proposed (no new fields; the old preferredDate and accept screen fall away) and awaits the owner's confirmation. Reminders are saved (see the Reminders sheet).</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Task 10a (app): ONE request form by extracting the shared "when and where" fields from TimeProposalForm (date, time, duration, on site, address prefilled from the saved account address, note) with native date and time pickers (Finding 2); remove the old preferredDate field from the form. The same shared fields serve the enter-a-time and counter screens.</t>
+          <t>Task 10a (app): ONE request form by extracting the shared "when and where" fields from TimeProposalForm (date, time, duration, on site, address prefilled from the saved account address, note) with native date and time pickers (Finding 2); (the old preferredDate field is already removed). The same shared fields serve the enter-a-time and counter screens.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Task 12: retire the old proposed-booking path for quotes, make the time required in the contract, delete preferredDate use and the AcceptQuoteScreen route, keep accept only for additional tasks; KEEP direct booking until Flow 2.</t>
+          <t>Task 12: retire the old proposed-booking path for quotes, make the time required in the contract, remove the AcceptQuoteScreen route (preferredDate is already gone), keep accept only for additional tasks; KEEP direct booking until Flow 2.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Task 12: retire the old proposed-booking path FOR QUOTES and make the time required in the contract (RequestInputSchema); remove the old preferredDate field from the app form (the database column stays for old requests until now) and the AcceptQuoteScreen route. Keep /quotes/[id]/accept for additional tasks only. KEEP direct booking (POST /bookings, the Book button for fixed-price services) until Flow 2 replaces it: two ways to propose a time on a booking exist knowingly until then.</t>
+          <t>Task 12: retire the old proposed-booking path FOR QUOTES and make the time required in the contract (RequestInputSchema); remove the AcceptQuoteScreen route (the old preferredDate field is already removed everywhere: DONE 1 Nov 2026, migration 0027). Keep /quotes/[id]/accept for additional tasks only. KEEP direct booking (POST /bookings, the Book button for fixed-price services) until Flow 2 replaces it: two ways to propose a time on a booking exist knowingly until then.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -4981,7 +4981,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>preferredDate (stop sending it now; the database column and its display stay for old requests until Task 12)</t>
+          <t>preferredDate: REMOVED on 1 Nov 2026 (column dropped by migration 0027, contract, server, data export, form, display and texts); nobody uses the app, so nothing is kept for old requests</t>
         </is>
       </c>
     </row>
@@ -5223,7 +5223,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>preferredDate in the contract input after old app builds are gone (Task 12)</t>
+          <t>Nothing left to remove: preferredDate is gone; the export now carries startAt, durationMin and onSite</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: the MVP workbook is one file updated in place (Reports/MVP Completion Tasks.xlsx), no dated copies
</commit_message>
<xml_diff>
--- a/Reports/MVP Completion Tasks.xlsx
+++ b/Reports/MVP Completion Tasks.xlsx
@@ -15,16 +15,18 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Owner actions" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reminders" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reuse map" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change log" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan'!$A$1:$I$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$H$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Plan'!$A$1:$J$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$1:$I$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Capstone scorecard'!$A$1:$E$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Owner decisions'!$A$1:$D$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Owner actions'!$A$1:$B$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Reminders'!$A$1:$D$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Reuse map'!$A$1:$D$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Change log'!$A$1:$D$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -46,7 +48,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -70,12 +72,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EDEDED"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -105,6 +102,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
@@ -121,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -129,7 +136,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -141,22 +163,10 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -663,7 +673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -675,6 +685,7 @@
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -723,6 +734,11 @@
           <t>Can run alongside</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -770,6 +786,11 @@
           <t>everything</t>
         </is>
       </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -817,6 +838,11 @@
           <t>0.3, 1.1</t>
         </is>
       </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -864,6 +890,11 @@
           <t>0.2, 1.1</t>
         </is>
       </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>Waiting for owner</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -911,6 +942,11 @@
           <t>0.2, 1.1</t>
         </is>
       </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>Waiting for owner</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -925,7 +961,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Confirm the reuse map for the app screens (Reuse map sheet) and the decision to keep direct booking until Flow 2; then update Tasks 10 to 12 of the Flow 1 plan as a reuse map (plan text only).</t>
+          <t>Confirm the reuse map for the app screens (Reuse map sheet); update Tasks 10 to 12 of the Flow 1 plan as a reuse map (plan text only). Note: the approved plan retires direct booking (the Book button opens the same request form), so the earlier suggestion to keep it until Flow 2 was dropped.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -956,6 +992,11 @@
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>0.2, 0.3</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1005,14 +1046,19 @@
           <t>everything</t>
         </is>
       </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>1.1</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>1 Finish Flow 1</t>
         </is>
@@ -1052,14 +1098,19 @@
           <t>0.x</t>
         </is>
       </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>Waiting for owner</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>1 Finish Flow 1</t>
         </is>
@@ -1095,14 +1146,19 @@
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>1.3</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>1 Finish Flow 1</t>
         </is>
@@ -1138,14 +1194,19 @@
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>1.4</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>1 Finish Flow 1</t>
         </is>
@@ -1181,14 +1242,19 @@
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>1.5</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>1 Finish Flow 1</t>
         </is>
@@ -1228,21 +1294,26 @@
           <t>1.6</t>
         </is>
       </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>1.6</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>1 Finish Flow 1</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Task 12: retire the old proposed-booking path for quotes, make the time required in the contract, remove the AcceptQuoteScreen route (preferredDate is already gone), keep accept only for additional tasks; KEEP direct booking until Flow 2.</t>
+          <t>Task 12: retire the old proposed-booking path for quotes, make the time required in the contract, remove the AcceptQuoteScreen route (preferredDate is already gone), keep accept only for additional tasks; The Book button opens the same request form; POST /bookings and BookScreen retire (instant booking returns with Flow 2).</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1275,14 +1346,19 @@
           <t>1.5</t>
         </is>
       </c>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>1.7</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>1 Finish Flow 1</t>
         </is>
@@ -1318,14 +1394,19 @@
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>1.8</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>1 Finish Flow 1</t>
         </is>
@@ -1365,14 +1446,19 @@
           <t>1.2-1.7</t>
         </is>
       </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>1.9</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>1 Finish Flow 1</t>
         </is>
@@ -1408,14 +1494,19 @@
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>1.10</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>1 Finish Flow 1</t>
         </is>
@@ -1451,14 +1542,19 @@
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="9" t="inlineStr">
         <is>
           <t>2.1</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>2 AI feature</t>
         </is>
@@ -1498,14 +1594,19 @@
           <t>Phase 1</t>
         </is>
       </c>
+      <c r="J18" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="9" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="9" t="inlineStr">
         <is>
           <t>2 AI feature</t>
         </is>
@@ -1541,14 +1642,19 @@
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" s="9" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>2 AI feature</t>
         </is>
@@ -1584,14 +1690,19 @@
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="9" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>2 AI feature</t>
         </is>
@@ -1627,14 +1738,19 @@
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>2 AI feature</t>
         </is>
@@ -1674,14 +1790,19 @@
           <t>2.3</t>
         </is>
       </c>
+      <c r="J22" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>2 AI feature</t>
         </is>
@@ -1717,14 +1838,19 @@
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>3.1</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>3 Security and compliance</t>
         </is>
@@ -1764,14 +1890,19 @@
           <t>3.2</t>
         </is>
       </c>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>3 Security and compliance</t>
         </is>
@@ -1811,14 +1942,19 @@
           <t>3.1</t>
         </is>
       </c>
+      <c r="J25" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>3.3</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>3 Security and compliance</t>
         </is>
@@ -1858,14 +1994,19 @@
           <t>2.x</t>
         </is>
       </c>
+      <c r="J26" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>3.4</t>
         </is>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>3 Security and compliance</t>
         </is>
@@ -1901,14 +2042,19 @@
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>3.5</t>
         </is>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>3 Security and compliance</t>
         </is>
@@ -1944,14 +2090,19 @@
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>4.1</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>4 Quality and evidence</t>
         </is>
@@ -1987,14 +2138,19 @@
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>4.2</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>4 Quality and evidence</t>
         </is>
@@ -2030,14 +2186,19 @@
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>4.3</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>4 Quality and evidence</t>
         </is>
@@ -2073,14 +2234,19 @@
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="A32" s="12" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B32" s="12" t="inlineStr">
         <is>
           <t>5 Presentation</t>
         </is>
@@ -2116,14 +2282,19 @@
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="A33" s="12" t="inlineStr">
         <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>5 Presentation</t>
         </is>
@@ -2159,14 +2330,19 @@
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="9" t="inlineStr">
+      <c r="A34" s="13" t="inlineStr">
         <is>
           <t>O.1</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>Owner actions (run in parallel from day 1)</t>
         </is>
@@ -2206,9 +2382,14 @@
           <t>Phases 1 to 3</t>
         </is>
       </c>
+      <c r="J34" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I34"/>
+  <autoFilter ref="A1:J34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2219,7 +2400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2230,6 +2411,7 @@
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2273,12 +2455,17 @@
           <t>Who</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="10" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -2311,6 +2498,11 @@
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Owner asks; Claude writes the note</t>
+        </is>
+      </c>
+      <c r="I2" s="6" t="inlineStr">
+        <is>
+          <t>Waiting for owner</t>
         </is>
       </c>
     </row>
@@ -2318,7 +2510,7 @@
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -2351,6 +2543,11 @@
       <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Both (owner decides provider and feature; planning started 1 Nov)</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -2358,7 +2555,7 @@
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -2391,6 +2588,11 @@
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Claude</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -2398,7 +2600,7 @@
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -2431,6 +2633,11 @@
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Owner merges; Claude prepares</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2438,7 +2645,7 @@
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -2471,6 +2678,11 @@
       <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Claude</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>Waiting for owner</t>
         </is>
       </c>
     </row>
@@ -2478,7 +2690,7 @@
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -2511,6 +2723,11 @@
       <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Claude</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>Waiting for owner</t>
         </is>
       </c>
     </row>
@@ -2518,7 +2735,7 @@
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -2551,6 +2768,11 @@
       <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Both</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2780,7 @@
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -2591,6 +2813,11 @@
       <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Claude (scan, code fixes); Owner (Vercel rules)</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2598,7 +2825,7 @@
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -2631,6 +2858,11 @@
       <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Owner (dashboard), Claude (scan)</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2638,7 +2870,7 @@
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -2671,6 +2903,11 @@
       <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Claude</t>
+        </is>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2678,7 +2915,7 @@
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -2711,6 +2948,11 @@
       <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Both</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2718,7 +2960,7 @@
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -2751,6 +2993,11 @@
       <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Owner tests, Claude fixes</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2758,7 +3005,7 @@
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -2791,6 +3038,11 @@
       <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Claude</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2798,7 +3050,7 @@
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -2831,6 +3083,11 @@
       <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Both</t>
+        </is>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2838,7 +3095,7 @@
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -2871,6 +3128,11 @@
       <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Claude, owner reads German</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
+        <is>
+          <t>Waiting for owner</t>
         </is>
       </c>
     </row>
@@ -2878,7 +3140,7 @@
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -2911,6 +3173,11 @@
       <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Claude</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2918,7 +3185,7 @@
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -2930,7 +3197,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Task 12: retire the old proposed-booking path FOR QUOTES and make the time required in the contract (RequestInputSchema); remove the AcceptQuoteScreen route (the old preferredDate field is already removed everywhere: DONE 1 Nov 2026, migration 0027). Keep /quotes/[id]/accept for additional tasks only. KEEP direct booking (POST /bookings, the Book button for fixed-price services) until Flow 2 replaces it: two ways to propose a time on a booking exist knowingly until then.</t>
+          <t>Task 12: retire the old proposed-booking path FOR QUOTES and make the time required in the contract (RequestInputSchema); remove the AcceptQuoteScreen route (the old preferredDate field is already removed everywhere: DONE 1 Nov 2026, migration 0027). Keep /quotes/[id]/accept for additional tasks only. The Book button for fixed-price services opens the same request form and POST /bookings plus BookScreen retire (as the approved plan says; instant booking returns with Flow 2). Old proposed rows are still answered until none exist.</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -2951,6 +3218,11 @@
       <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Claude</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2958,7 +3230,7 @@
       <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -2991,6 +3263,11 @@
       <c r="H19" s="2" t="inlineStr">
         <is>
           <t>Claude</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -2998,7 +3275,7 @@
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3031,6 +3308,11 @@
       <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Owner</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3320,7 @@
       <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3071,6 +3353,11 @@
       <c r="H21" s="2" t="inlineStr">
         <is>
           <t>Both</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -3078,7 +3365,7 @@
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3111,6 +3398,11 @@
       <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Owner</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3118,7 +3410,7 @@
       <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="11" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3151,6 +3443,11 @@
       <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Both</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3455,7 @@
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3191,6 +3488,11 @@
       <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Claude</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3500,7 @@
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="11" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3231,6 +3533,11 @@
       <c r="H25" s="2" t="inlineStr">
         <is>
           <t>Both</t>
+        </is>
+      </c>
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3545,7 @@
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3271,6 +3578,11 @@
       <c r="H26" s="2" t="inlineStr">
         <is>
           <t>Owner</t>
+        </is>
+      </c>
+      <c r="I26" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3278,7 +3590,7 @@
       <c r="A27" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3311,6 +3623,11 @@
       <c r="H27" s="2" t="inlineStr">
         <is>
           <t>Claude</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3318,7 +3635,7 @@
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3351,6 +3668,11 @@
       <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Owner</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3358,7 +3680,7 @@
       <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3391,6 +3713,11 @@
       <c r="H29" s="2" t="inlineStr">
         <is>
           <t>Claude</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3398,7 +3725,7 @@
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3431,6 +3758,11 @@
       <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Owner</t>
+        </is>
+      </c>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3438,7 +3770,7 @@
       <c r="A31" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3471,6 +3803,11 @@
       <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Owner</t>
+        </is>
+      </c>
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3478,7 +3815,7 @@
       <c r="A32" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3511,6 +3848,11 @@
       <c r="H32" s="2" t="inlineStr">
         <is>
           <t>Claude</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3518,7 +3860,7 @@
       <c r="A33" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3551,6 +3893,11 @@
       <c r="H33" s="2" t="inlineStr">
         <is>
           <t>Claude</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3558,7 +3905,7 @@
       <c r="A34" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3591,6 +3938,11 @@
       <c r="H34" s="2" t="inlineStr">
         <is>
           <t>Owner</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3598,7 +3950,7 @@
       <c r="A35" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3631,6 +3983,11 @@
       <c r="H35" s="2" t="inlineStr">
         <is>
           <t>Both</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3638,7 +3995,7 @@
       <c r="A36" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="8" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3671,6 +4028,11 @@
       <c r="H36" s="2" t="inlineStr">
         <is>
           <t>Claude</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3678,7 +4040,7 @@
       <c r="A37" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3711,6 +4073,11 @@
       <c r="H37" s="2" t="inlineStr">
         <is>
           <t>Both</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3718,7 +4085,7 @@
       <c r="A38" s="2" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="7" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3751,6 +4118,11 @@
       <c r="H38" s="2" t="inlineStr">
         <is>
           <t>Owner</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3758,7 +4130,7 @@
       <c r="A39" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="7" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3791,6 +4163,11 @@
       <c r="H39" s="2" t="inlineStr">
         <is>
           <t>Owner</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3798,7 +4175,7 @@
       <c r="A40" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="7" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3831,6 +4208,11 @@
       <c r="H40" s="2" t="inlineStr">
         <is>
           <t>Both</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3838,7 +4220,7 @@
       <c r="A41" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3871,6 +4253,11 @@
       <c r="H41" s="2" t="inlineStr">
         <is>
           <t>Owner</t>
+        </is>
+      </c>
+      <c r="I41" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
@@ -3878,7 +4265,7 @@
       <c r="A42" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="7" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3913,9 +4300,14 @@
           <t>Both</t>
         </is>
       </c>
+      <c r="I42" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H42"/>
+  <autoFilter ref="A1:I42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3974,7 +4366,7 @@
           <t>Completeness and functionality; runs at a live Vercel URL or on a phone</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
@@ -4001,7 +4393,7 @@
           <t>User interface and interaction quality</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
@@ -4028,7 +4420,7 @@
           <t>Clear README.md with a goal / problem / how-it-works paragraph</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
@@ -4055,7 +4447,7 @@
           <t>Course stack: Next.js, Supabase Auth and RLS, Vercel</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Met</t>
         </is>
@@ -4082,7 +4474,7 @@
           <t>CLAUDE.md</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Not met</t>
         </is>
@@ -4109,7 +4501,7 @@
           <t>At least one skill, slash command or subagent used</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
@@ -4136,7 +4528,7 @@
           <t>At least one pull request reviewed before merging</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
@@ -4163,7 +4555,7 @@
           <t>Secrets out of the repo, server side only</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Met</t>
         </is>
@@ -4190,7 +4582,7 @@
           <t>Row-level security on every table holding user data</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Met</t>
         </is>
@@ -4217,7 +4609,7 @@
           <t>A /security-scan pass</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
@@ -4244,7 +4636,7 @@
           <t>AI-generated content disclosed (Article 50)</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
@@ -4271,7 +4663,7 @@
           <t>Working "delete my data" route (GDPR)</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Partly</t>
         </is>
@@ -4298,7 +4690,7 @@
           <t>SCR or SMART framing, clear explanation</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Not met</t>
         </is>
@@ -4325,7 +4717,7 @@
           <t>Showcase upload and 10 + 5 minute presentation</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Not met</t>
         </is>
@@ -5152,12 +5544,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>KEEP until Flow 2 (instant booking) replaces it</t>
+          <t>The Book button opens the SAME request form with the service chosen (as the approved plan says: one flow); instant booking returns with Flow 2</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Two ways to propose a time on a booking coexist knowingly (proposed/counter vs awaiting-time/pending time); unify in Flow 2</t>
+          <t>BookScreen and POST /bookings retire in Task 12; old proposed rows are still answered until none exist (known leftover)</t>
         </is>
       </c>
     </row>
@@ -5231,4 +5623,441 @@
   <autoFilter ref="A1:D13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="120" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>What changed</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Plan steps / tasks affected</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-02 00:03</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>e5717b3</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Workbook is now one file, Reports/MVP Completion Tasks.xlsx, updated in place (owner rule 2 Nov 2026); written now with the current state (steps 1.3 to 1.5)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 23:59</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>9fb1759</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Code review of PR 54: 4 findings fixed, 5 rejected after checking; record posted on the PR</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 23:15</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>7022f7e</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Steps 1.4 and 1.5 on PR #54: customer confirms a quote directly, Decline offers the chat first, request shows time and place, awaiting-time enter/confirm agreed time; quote lists with PDF link in the account tab</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>step 1.4 Done, step 1.5 Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 22:51</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>ad81df8</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Step 1.3: provider answer form with pickers, prefill from the request and the Date and time confirmed switch; rule recorded: PRs without code changes are not counted for the workbook</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>step 1.3 Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 22:44</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>5a66db1</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>AI plan approved by the owner (1 Nov 2026)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>step 0.2 Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 22:41</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>53b1beb</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>AI plan written (docs/superpowers/plans/2026-11-01-ai-document-check.md) with the owner decisions: human sees only ID problems plus 10% sample, 30-day ID deletion, only verdict and reason stored</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>step 0.2 Waiting for owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 22:26</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>3c08c72</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Production migrations 0024-0027 applied by the owner (1 Nov 2026); #49 code confirmed live (quotes route answers 401); live site probes fine</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 21:52</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>53b1beb</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>PRs 48, 49 and 51 merged (51 carries the #50 content, which had been merged into the #49 branch by mistake); step 1.2 on main</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>step 1.2 Done, merged PR #48, merged PR #49, merged PR #51</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 18:29</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>64bafa9</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Code review of PR 50 (/code-review): 7 findings fixed (iPhone picker default and Done button, past time today refused, remote only for remote providers, address prefill once and shared with the time proposal form, 24-hour display); the typed fields of the send-quote form are step 1.3. Review record posted on PR 50.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 18:17</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2024ae1</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Code review of PR 49 (/code-review): fixed the sweep clock and count, on-demand PDF storing, tracker script robustness; documented the deploy order of migration 0027 (apply after the code); rejected 3 findings (dense versions, trader retention, stricter checks on entering a time). Review record posted on PR 49.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 17:07</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>b460758</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.2 (Task 10a, Finding 2): one shared set of when-and-where fields (WhenWhereFields, buildProposal) with native date and time pickers, used by the request form and the time proposal form; the request form now sends start, duration, place, address (prefilled from the saved account address) and note, so the app works with the server again. New native dependency @react-native-community/datetimepicker: a new Android build is needed. Owner: review and merge PR 50 (stacked on PR 49), then make the build and test on the phone.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>step 1.2 Waiting for owner, task 3 In progress, task 20 In progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 16:55</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>0f16a5a</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>CI of PR 48 failed on booking-notifications: the test compared a date without leading zeros (1.1.2027) with the email's 01.01.2027; it failed because today plus 60 days is 1 January. Fixed in the test on both branches (PR 48 and PR 49); my earlier time-of-day explanation was incomplete.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 16:04</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>4373a83</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Phase 0.6 done: review records posted as comments on 12 merged PRs (2, 5, 11, 14, 15, 16, 29, 30, 35, 36, 37, 38) copied from the written reports, and on PRs 47 and 48 (code review of this session). Not posted on 25, 27, 28 and 18 to 20: the reports hold only partial or no code-review lines for them. /code-review 48 was run; findings fixed in PR 48. Still for the owner: submit a GitHub review (Approve) on PR 48 and PR 49 before merging.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>step 0.6 Done, task 7 In progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 16:01</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>ec300ca</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>PR 47 was merged by the owner at its earlier head (2e093d6); the later work (tasks 6b to 9, preferredDate removal, review fixes, tracker) is in the new PR 49 (branch merged with main, conflicts resolved for the branch). PR 48 (CLAUDE.md, .claude folder, RLS note) still open; review records posted on PRs 47 and 48. Production needs migrations 0024 to 0026 (and 0027 with PR 49) - owner to check.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>step 1.1 Waiting for owner, task 15 Waiting for owner, merged PR #47</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 15:49</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>ad03c64</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Review of PR 47 (/code-review): fixed the missing-document sweep and revision numbering, account deletion and data export for quote documents, VAT arithmetic in cents, the checks and the clash check when a time is entered, a stale comment. Rejected or documented: dropped preferredDate column (owner decision), stand-in start time (README), quote expiry cap, no reminder for awaiting-time expiry. Tracker rule changed: the workbook is written after every 2 merged PRs.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>step 0.1 In progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 15:00</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>d325b15</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Phase 1.1 (Task 9): notice wording for the one-flow request in German and English (in-app, push, email); the sweep test no longer depends on the time of day (it failed after midday, also without these changes). The owner should read the German texts. Added the /update-mvp-report command.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>step 1.1 Done, step 0.1 In progress, task 15 Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 14:49</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>e971d62</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Phase 0.3 and 0.4 on PR #48 (branch chore/claude-folder): CLAUDE.md, the rls-check agent, the /test-report command, project .claude folder with README, RLS and auth evidence note, README section on how the project is built with Claude Code. Waiting for the owner: run /code-review --comment on PR #48, submit a GitHub review, merge.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>step 0.3 Waiting for owner, step 0.4 Waiting for owner, task 1 Waiting for owner, task 5 Waiting for owner, task 6 Waiting for owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 14:45</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>ab7813f</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Phase 0.5: Tasks 10 to 12 of the Flow 1 plan now carry the confirmed reuse map; the plan keeps the approved one-flow rule (the Book button opens the request form, direct booking retires in Task 12); tracked-update tooling (docs/mvp) added</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>step 0.5 Done, step 0.1 In progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-01 12:00</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>1f9423a</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Baseline before the tracked updates: server side of Flow 1 built (tasks 1 to 8 incl. 6a, 6b, 7), the old preferredDate field removed everywhere (migration 0027), the .claude folder pushed on branch chore/claude-folder, owner decisions recorded (Neon approved; AI feature direction).</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>step 0.1 In progress, step 0.2 In progress, step 0.3 In progress, task 1 In progress</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D20"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>